<commit_message>
Improve parser validation and documentation
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -531,7 +531,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-08-12T23:26:48+05:00</t>
+          <t>2026-08-12T23:43:32+05:00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -579,7 +579,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-08-12T23:26:48+05:00</t>
+          <t>2026-08-12T23:43:32+05:00</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-08-12T23:26:48+05:00</t>
+          <t>2026-08-12T23:43:32+05:00</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-12T23:26:48+05:00</t>
+          <t>2026-08-12T23:43:32+05:00</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-12T23:26:48+05:00</t>
+          <t>2026-08-12T23:43:32+05:00</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-12T23:26:48+05:00</t>
+          <t>2026-08-12T23:43:32+05:00</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-12T23:26:48+05:00</t>
+          <t>2026-08-12T23:43:32+05:00</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-12T23:26:48+05:00</t>
+          <t>2026-08-12T23:43:32+05:00</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-12T23:26:48+05:00</t>
+          <t>2026-08-12T23:43:32+05:00</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-12T23:26:48+05:00</t>
+          <t>2026-08-12T23:43:32+05:00</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">

</xml_diff>